<commit_message>
docs: 更新 README 与新增 NovaSpark2.0 引导脚本
</commit_message>
<xml_diff>
--- a/Assets/Samples/GameLoginDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/GameLoginDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
   <si>
     <t>##comment</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t>/v1/user/delete</t>
+  </si>
+  <si>
+    <t>GameAccountBindResolve</t>
+  </si>
+  <si>
+    <t>绑定切换（绑定冲突时的二选一方案）</t>
+  </si>
+  <si>
+    <t>/v1/account/bind/resolve</t>
   </si>
   <si>
     <t>TGAServerUrl</t>
@@ -1165,7 +1174,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U43"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -1324,38 +1333,70 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8" t="s">
+    <row r="7" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A7" s="1"/>
+      <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+    </row>
+    <row r="8" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A8" s="7"/>
+      <c r="B8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="8"/>
-      <c r="S7" s="8"/>
-      <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
+      <c r="C8" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
     </row>
-    <row r="8" ht="22" customHeight="1"/>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1"/>
     <row r="11" ht="22" customHeight="1"/>
@@ -1391,6 +1432,7 @@
     <row r="41" ht="22" customHeight="1"/>
     <row r="42" ht="22" customHeight="1"/>
     <row r="43" ht="22" customHeight="1"/>
+    <row r="44" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
chore: publish upm packages
Published packages:
- com.solotopia.nova.framework@0.5.33
- com.solotopia.nova.framework.kit.network.gamebind@0.0.1
- com.solotopia.nova.framework.kit.network.gamelogin@0.0.8
- com.solotopia.nova.framework.kit.network.gamesave@0.0.15
</commit_message>
<xml_diff>
--- a/Assets/Samples/GameLoginDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/GameLoginDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
   <si>
     <t>##comment</t>
   </si>
@@ -98,10 +98,28 @@
     <t>/v1/user/delete</t>
   </si>
   <si>
+    <t>GameAccountBind</t>
+  </si>
+  <si>
+    <t>绑定</t>
+  </si>
+  <si>
+    <t>/v1/account/bind</t>
+  </si>
+  <si>
+    <t>GameAccountBindConflict</t>
+  </si>
+  <si>
+    <t>绑定冲突查询</t>
+  </si>
+  <si>
+    <t>/v1/account/bind/conflict</t>
+  </si>
+  <si>
     <t>GameAccountBindResolve</t>
   </si>
   <si>
-    <t>绑定切换（绑定冲突时的二选一方案）</t>
+    <t>绑定裁决</t>
   </si>
   <si>
     <t>/v1/account/bind/resolve</t>
@@ -1174,7 +1192,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U44"/>
+  <dimension ref="A1:U46"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -1366,39 +1384,103 @@
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
     </row>
-    <row r="8" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8" t="s">
+    <row r="8" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A8" s="1"/>
+      <c r="B8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
+    </row>
+    <row r="9" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A9" s="1"/>
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
+      <c r="C9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
     </row>
-    <row r="9" ht="22" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1"/>
+    <row r="10" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A10" s="7"/>
+      <c r="B10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+    </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1"/>
@@ -1433,6 +1515,8 @@
     <row r="42" ht="22" customHeight="1"/>
     <row r="43" ht="22" customHeight="1"/>
     <row r="44" ht="22" customHeight="1"/>
+    <row r="45" ht="22" customHeight="1"/>
+    <row r="46" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>